<commit_message>
added a4 4x4 labels on pdf
</commit_message>
<xml_diff>
--- a/backend/shipping/data/failure.xlsx
+++ b/backend/shipping/data/failure.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Row No</t>
   </si>
@@ -21,6 +21,30 @@
   </si>
   <si>
     <t>Error Message</t>
+  </si>
+  <si>
+    <t>CR176996649132</t>
+  </si>
+  <si>
+    <t>Waybill already genereated for this CreditReferenceNo. Waybill No : 90001537150 Dest Area :DEL Dest Scrcd :NRA</t>
+  </si>
+  <si>
+    <t>CR176996649134</t>
+  </si>
+  <si>
+    <t>Waybill already genereated for this CreditReferenceNo. Waybill No : 90001537161 Dest Area :DEL Dest Scrcd :NRA</t>
+  </si>
+  <si>
+    <t>CR176996649135</t>
+  </si>
+  <si>
+    <t>Collectable Amount can not be zero for COD/DOD/DODFOD</t>
+  </si>
+  <si>
+    <t>CR176996649136</t>
+  </si>
+  <si>
+    <t>Waybill already genereated for this CreditReferenceNo. Waybill No : 90001537172 Dest Area :DEL Dest Scrcd :NRA</t>
   </si>
 </sst>
 </file>
@@ -65,7 +89,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -79,6 +103,50 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Added bulk import dim sheet
</commit_message>
<xml_diff>
--- a/backend/shipping/data/failure.xlsx
+++ b/backend/shipping/data/failure.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Row No</t>
   </si>
@@ -23,28 +23,22 @@
     <t>Error Message</t>
   </si>
   <si>
-    <t>CR176996649132</t>
+    <t>CR940120</t>
   </si>
   <si>
-    <t>Waybill already genereated for this CreditReferenceNo. Waybill No : 90001537150 Dest Area :DEL Dest Scrcd :NRA</t>
+    <t>Waybill already genereated for this CreditReferenceNo. Waybill No : 77707350033 Dest Area :DEL Dest Scrcd :NRA</t>
   </si>
   <si>
-    <t>CR176996649134</t>
+    <t>CR940122</t>
   </si>
   <si>
-    <t>Waybill already genereated for this CreditReferenceNo. Waybill No : 90001537161 Dest Area :DEL Dest Scrcd :NRA</t>
+    <t>Waybill already genereated for this CreditReferenceNo. Waybill No : 68503657482 Dest Area :DEL Dest Scrcd :WDW</t>
   </si>
   <si>
-    <t>CR176996649135</t>
+    <t>CR940123</t>
   </si>
   <si>
-    <t>Collectable Amount can not be zero for COD/DOD/DODFOD</t>
-  </si>
-  <si>
-    <t>CR176996649136</t>
-  </si>
-  <si>
-    <t>Waybill already genereated for this CreditReferenceNo. Waybill No : 90001537172 Dest Area :DEL Dest Scrcd :NRA</t>
+    <t>Collectable Amount is not applicable for other than COD/DOD/DODFOD shipments</t>
   </si>
 </sst>
 </file>
@@ -89,7 +83,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -136,17 +130,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n" s="0">
-        <v>5.0</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>